<commit_message>
feat: complete Teacher Management & RBAC system with secure API ownership checks
</commit_message>
<xml_diff>
--- a/Stdlist.xlsx
+++ b/Stdlist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Apps\Classtest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC03F88D-62FC-4E6D-88CB-37D5BB8CAC09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F01EF648-AB98-4526-9C7B-E2D8027FD309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{360468C9-B75F-4461-9633-B4866D871250}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{664C5D66-FD01-49D7-B134-66D1304C9B64}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="180">
   <si>
     <t>AADARSH</t>
   </si>
@@ -172,21 +172,21 @@
     <t>YASHVI YADAV</t>
   </si>
   <si>
+    <t>class</t>
+  </si>
+  <si>
+    <t>section</t>
+  </si>
+  <si>
+    <t>admno</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
     <t>A</t>
   </si>
   <si>
-    <t>admno</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>class</t>
-  </si>
-  <si>
-    <t>section</t>
-  </si>
-  <si>
     <t>AABHAS BANSAL</t>
   </si>
   <si>
@@ -314,23 +314,276 @@
   </si>
   <si>
     <t>YAJURV</t>
+  </si>
+  <si>
+    <t>AARAV PATEL</t>
+  </si>
+  <si>
+    <t>AARIV TUDU</t>
+  </si>
+  <si>
+    <t>ABHAY CHAUDHARY</t>
+  </si>
+  <si>
+    <t>ABHAY SINGH</t>
+  </si>
+  <si>
+    <t>ADITI JANGRA</t>
+  </si>
+  <si>
+    <t>ADITI PYASI</t>
+  </si>
+  <si>
+    <t>ADITYA</t>
+  </si>
+  <si>
+    <t>ADITYA CHAUDHARY</t>
+  </si>
+  <si>
+    <t>AMITA VERMA</t>
+  </si>
+  <si>
+    <t>ANANTJIT MISHRA</t>
+  </si>
+  <si>
+    <t>ANKITA ACHARYA</t>
+  </si>
+  <si>
+    <t>ANUJ CHAUDHARY</t>
+  </si>
+  <si>
+    <t>ARADHYA SINGH</t>
+  </si>
+  <si>
+    <t>ATASI DALAL</t>
+  </si>
+  <si>
+    <t>ATIKSH RANA</t>
+  </si>
+  <si>
+    <t>ATUL KUMAR</t>
+  </si>
+  <si>
+    <t>AYUSH KUMAR</t>
+  </si>
+  <si>
+    <t>DEV PRATAP SINGH</t>
+  </si>
+  <si>
+    <t>DEVANSH YADAV</t>
+  </si>
+  <si>
+    <t>DEVRAJ CHAUDHARY</t>
+  </si>
+  <si>
+    <t>DIVYA YADAV</t>
+  </si>
+  <si>
+    <t>GAURAVI KORANGA</t>
+  </si>
+  <si>
+    <t>GUNJIT CHAUDHARY</t>
+  </si>
+  <si>
+    <t>JAHNAVI ANAND</t>
+  </si>
+  <si>
+    <t>KANISHKA SAINI</t>
+  </si>
+  <si>
+    <t>KARISHMA BAGHEL</t>
+  </si>
+  <si>
+    <t>KRATIKA CHAUDHARY</t>
+  </si>
+  <si>
+    <t>KUNJ VERMA</t>
+  </si>
+  <si>
+    <t>MADHAV CHAUDHARY</t>
+  </si>
+  <si>
+    <t>MAYANK CHAUDHARY</t>
+  </si>
+  <si>
+    <t>MRIDUL SHARMA</t>
+  </si>
+  <si>
+    <t>NIDHI</t>
+  </si>
+  <si>
+    <t>PRIYAL SINGH</t>
+  </si>
+  <si>
+    <t>PRIYANSHU VERMA</t>
+  </si>
+  <si>
+    <t>R CHHARVY REDDY</t>
+  </si>
+  <si>
+    <t>RAJ SINGH</t>
+  </si>
+  <si>
+    <t>RIDHI</t>
+  </si>
+  <si>
+    <t>RUDRESH UPADHYAY</t>
+  </si>
+  <si>
+    <t>SARANSH SINGH</t>
+  </si>
+  <si>
+    <t>SHAMBHAVI SHAH</t>
+  </si>
+  <si>
+    <t>SHIVANYA SISODIA</t>
+  </si>
+  <si>
+    <t>SUHANA RAWAT</t>
+  </si>
+  <si>
+    <t>VIRAT TOMAR</t>
+  </si>
+  <si>
+    <t>VIVEK RAJ</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>AAKARSH RANJAN</t>
+  </si>
+  <si>
+    <t>AARAV</t>
+  </si>
+  <si>
+    <t>ABHINAV KUMAR SINGH</t>
+  </si>
+  <si>
+    <t>ANISHA DIXIT</t>
+  </si>
+  <si>
+    <t>ANKIT VASHISTHA</t>
+  </si>
+  <si>
+    <t>ANNU PALHAWAT</t>
+  </si>
+  <si>
+    <t>ANSH</t>
+  </si>
+  <si>
+    <t>ANUSHKA SINGH</t>
+  </si>
+  <si>
+    <t>ANYA SINGH</t>
+  </si>
+  <si>
+    <t>AYANSH TRIPATHI</t>
+  </si>
+  <si>
+    <t>DARSHIKA</t>
+  </si>
+  <si>
+    <t>DIPTI</t>
+  </si>
+  <si>
+    <t>DIVYANSHI DESHWAR</t>
+  </si>
+  <si>
+    <t>GARVIT GUPTA</t>
+  </si>
+  <si>
+    <t>HRIDHANSH CHAUDHARY</t>
+  </si>
+  <si>
+    <t>ISHITA DUBEY</t>
+  </si>
+  <si>
+    <t>JASMITH SINGH</t>
+  </si>
+  <si>
+    <t>JEEVA CHOUDHARY</t>
+  </si>
+  <si>
+    <t>JOSHITA SINGH</t>
+  </si>
+  <si>
+    <t>KESHAV KUMAR SHARMA</t>
+  </si>
+  <si>
+    <t>KHUSHI</t>
+  </si>
+  <si>
+    <t>KUNWAR ABHAY PRATAP SINGH</t>
+  </si>
+  <si>
+    <t>MANAN DHAKAR</t>
+  </si>
+  <si>
+    <t>MUDIT SIKARWAR</t>
+  </si>
+  <si>
+    <t>NIRBHAY</t>
+  </si>
+  <si>
+    <t>NISHANT SIKARWAR</t>
+  </si>
+  <si>
+    <t>OJASVI SINGH</t>
+  </si>
+  <si>
+    <t>PARI SISODIA</t>
+  </si>
+  <si>
+    <t>PRABHAV VAISHNAV</t>
+  </si>
+  <si>
+    <t>PRAGATI SHAKYA</t>
+  </si>
+  <si>
+    <t>PRAHALAD SINGH RAWAT</t>
+  </si>
+  <si>
+    <t>RADHIKA</t>
+  </si>
+  <si>
+    <t>RISHI</t>
+  </si>
+  <si>
+    <t>SAKSHI KUMARI</t>
+  </si>
+  <si>
+    <t>SHAURYA ANAND</t>
+  </si>
+  <si>
+    <t>TARUN</t>
+  </si>
+  <si>
+    <t>TARUN SHARMA</t>
+  </si>
+  <si>
+    <t>VANSH KASHYAP</t>
+  </si>
+  <si>
+    <t>VIHAAN SAHU</t>
+  </si>
+  <si>
+    <t>VISHAL</t>
+  </si>
+  <si>
+    <t>YUGAL</t>
+  </si>
+  <si>
+    <t>C</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -342,6 +595,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -382,7 +640,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -696,1261 +954,2451 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFDE53A8-B336-4C9B-AC2C-CD7784BD64DE}">
-  <dimension ref="A1:D89"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{298C44AE-6B8F-48A6-B234-EB7B9FC5D6A2}">
+  <dimension ref="A1:D174"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1">
         <v>9512</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C2">
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="1">
         <v>11648</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C3">
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1">
         <v>9646</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C4">
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="1">
         <v>9577</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C5">
         <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="1">
         <v>9931</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C6">
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1">
         <v>11650</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C7">
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="1">
         <v>9511</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C8">
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="1">
         <v>9837</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C9">
         <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="1">
         <v>10223</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C10">
         <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="1">
         <v>9809</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C11">
         <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="1">
         <v>9765</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="1">
         <v>11150</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C13">
         <v>6</v>
       </c>
       <c r="D13" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="1">
         <v>10334</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C14">
         <v>6</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="1">
         <v>9473</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C15">
         <v>6</v>
       </c>
       <c r="D15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="1">
         <v>9452</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C16">
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="1">
         <v>10178</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C17">
         <v>6</v>
       </c>
       <c r="D17" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="1">
         <v>11598</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C18">
         <v>6</v>
       </c>
       <c r="D18" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="1">
         <v>10021</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C19">
         <v>6</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="1">
         <v>9481</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C20">
         <v>6</v>
       </c>
       <c r="D20" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="1">
         <v>9565</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C21">
         <v>6</v>
       </c>
       <c r="D21" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="1">
         <v>9463</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="1">
         <v>10137</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C23">
         <v>6</v>
       </c>
       <c r="D23" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="1">
         <v>9477</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C24">
         <v>6</v>
       </c>
       <c r="D24" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="1">
         <v>9465</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C25">
         <v>6</v>
       </c>
       <c r="D25" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="1">
         <v>10340</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C26">
         <v>6</v>
       </c>
       <c r="D26" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="1">
         <v>10159</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C27">
         <v>6</v>
       </c>
       <c r="D27" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="1">
         <v>10690</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C28">
         <v>6</v>
       </c>
       <c r="D28" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="1">
         <v>9456</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C29">
         <v>6</v>
       </c>
       <c r="D29" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="1">
         <v>11361</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C30">
         <v>6</v>
       </c>
       <c r="D30" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="1">
         <v>9515</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C31">
         <v>6</v>
       </c>
       <c r="D31" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="1">
         <v>11268</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C32">
         <v>6</v>
       </c>
       <c r="D32" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="1">
         <v>9630</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C33">
         <v>6</v>
       </c>
       <c r="D33" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="1">
         <v>9472</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C34">
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="1">
         <v>10089</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C35">
         <v>6</v>
       </c>
       <c r="D35" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="1">
         <v>9674</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="1" t="s">
         <v>34</v>
       </c>
       <c r="C36">
         <v>6</v>
       </c>
       <c r="D36" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="1">
         <v>11162</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C37">
         <v>6</v>
       </c>
       <c r="D37" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="1">
         <v>9460</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C38">
         <v>6</v>
       </c>
       <c r="D38" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="1">
         <v>9459</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C39">
         <v>6</v>
       </c>
       <c r="D39" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="1">
         <v>9977</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C40">
         <v>6</v>
       </c>
       <c r="D40" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="1">
         <v>9491</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C41">
         <v>6</v>
       </c>
       <c r="D41" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="1">
         <v>9997</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C42">
         <v>6</v>
       </c>
       <c r="D42" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="1">
         <v>10004</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C43">
         <v>6</v>
       </c>
       <c r="D43" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="1">
         <v>9484</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C44">
         <v>6</v>
       </c>
       <c r="D44" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="1">
         <v>11468</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C45">
         <v>6</v>
       </c>
       <c r="D45" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="1">
         <v>11658</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C46">
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="1">
         <v>10310</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="1">
         <v>10645</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C48">
         <v>7</v>
       </c>
       <c r="D48" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" s="1">
         <v>10266</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="1" t="s">
         <v>52</v>
       </c>
       <c r="C49">
         <v>7</v>
       </c>
       <c r="D49" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="1">
         <v>9231</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="1" t="s">
         <v>53</v>
       </c>
       <c r="C50">
         <v>7</v>
       </c>
       <c r="D50" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" s="1">
         <v>11040</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C51">
         <v>7</v>
       </c>
       <c r="D51" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="1">
         <v>10795</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="1" t="s">
         <v>55</v>
       </c>
       <c r="C52">
         <v>7</v>
       </c>
       <c r="D52" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="1">
         <v>10474</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C53">
         <v>7</v>
       </c>
       <c r="D53" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="1">
         <v>9333</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="1" t="s">
         <v>57</v>
       </c>
       <c r="C54">
         <v>7</v>
       </c>
       <c r="D54" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" s="1">
         <v>9280</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" s="1" t="s">
         <v>58</v>
       </c>
       <c r="C55">
         <v>7</v>
       </c>
       <c r="D55" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="1">
         <v>9241</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="1" t="s">
         <v>59</v>
       </c>
       <c r="C56">
         <v>7</v>
       </c>
       <c r="D56" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="1">
         <v>9440</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" s="1" t="s">
         <v>60</v>
       </c>
       <c r="C57">
         <v>7</v>
       </c>
       <c r="D57" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="1">
         <v>9306</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="1" t="s">
         <v>61</v>
       </c>
       <c r="C58">
         <v>7</v>
       </c>
       <c r="D58" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="1">
         <v>10114</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C59">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="1">
         <v>9213</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="1" t="s">
         <v>63</v>
       </c>
       <c r="C60">
         <v>7</v>
       </c>
       <c r="D60" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="1">
         <v>11163</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C61">
         <v>7</v>
       </c>
       <c r="D61" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="1">
         <v>10364</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="1" t="s">
         <v>65</v>
       </c>
       <c r="C62">
         <v>7</v>
       </c>
       <c r="D62" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="1">
         <v>9264</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B63" s="1" t="s">
         <v>66</v>
       </c>
       <c r="C63">
         <v>7</v>
       </c>
       <c r="D63" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="1">
         <v>9254</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="1" t="s">
         <v>67</v>
       </c>
       <c r="C64">
         <v>7</v>
       </c>
       <c r="D64" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="1">
         <v>9206</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="1" t="s">
         <v>68</v>
       </c>
       <c r="C65">
         <v>7</v>
       </c>
       <c r="D65" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="1">
         <v>9215</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="1" t="s">
         <v>69</v>
       </c>
       <c r="C66">
         <v>7</v>
       </c>
       <c r="D66" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="1">
         <v>11248</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="1" t="s">
         <v>70</v>
       </c>
       <c r="C67">
         <v>7</v>
       </c>
       <c r="D67" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="1">
         <v>9204</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="1" t="s">
         <v>71</v>
       </c>
       <c r="C68">
         <v>7</v>
       </c>
       <c r="D68" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" s="1">
         <v>9933</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="1" t="s">
         <v>72</v>
       </c>
       <c r="C69">
         <v>7</v>
       </c>
       <c r="D69" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="1">
         <v>11529</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="1" t="s">
         <v>73</v>
       </c>
       <c r="C70">
         <v>7</v>
       </c>
       <c r="D70" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="1">
         <v>10772</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" s="1" t="s">
         <v>74</v>
       </c>
       <c r="C71">
         <v>7</v>
       </c>
       <c r="D71" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" s="1">
         <v>9302</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" s="1" t="s">
         <v>75</v>
       </c>
       <c r="C72">
         <v>7</v>
       </c>
       <c r="D72" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" s="1">
         <v>9207</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" s="1" t="s">
         <v>76</v>
       </c>
       <c r="C73">
         <v>7</v>
       </c>
       <c r="D73" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74" s="1">
         <v>11050</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="1" t="s">
         <v>77</v>
       </c>
       <c r="C74">
         <v>7</v>
       </c>
       <c r="D74" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
+      <c r="A75" s="1">
         <v>9240</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C75">
         <v>7</v>
       </c>
       <c r="D75" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
+      <c r="A76" s="1">
         <v>9222</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" s="1" t="s">
         <v>79</v>
       </c>
       <c r="C76">
         <v>7</v>
       </c>
       <c r="D76" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
+      <c r="A77" s="1">
         <v>9223</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C77">
         <v>7</v>
       </c>
       <c r="D77" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="A78" s="1">
         <v>11292</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" s="1" t="s">
         <v>81</v>
       </c>
       <c r="C78">
         <v>7</v>
       </c>
       <c r="D78" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="A79" s="1">
         <v>11635</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B79" s="1" t="s">
         <v>82</v>
       </c>
       <c r="C79">
         <v>7</v>
       </c>
       <c r="D79" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80" s="1">
         <v>11271</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B80" s="1" t="s">
         <v>83</v>
       </c>
       <c r="C80">
         <v>7</v>
       </c>
       <c r="D80" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
+      <c r="A81" s="1">
         <v>10468</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="B81" s="1" t="s">
         <v>84</v>
       </c>
       <c r="C81">
         <v>7</v>
       </c>
       <c r="D81" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4">
+      <c r="A82" s="1">
         <v>9312</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" s="1" t="s">
         <v>85</v>
       </c>
       <c r="C82">
         <v>7</v>
       </c>
       <c r="D82" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
+      <c r="A83" s="1">
         <v>11035</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B83" s="1" t="s">
         <v>86</v>
       </c>
       <c r="C83">
         <v>7</v>
       </c>
       <c r="D83" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
+      <c r="A84" s="1">
         <v>9963</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="B84" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C84">
         <v>7</v>
       </c>
       <c r="D84" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
+      <c r="A85" s="1">
         <v>9212</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="B85" s="1" t="s">
         <v>88</v>
       </c>
       <c r="C85">
         <v>7</v>
       </c>
       <c r="D85" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
+      <c r="A86" s="1">
         <v>9313</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B86" s="1" t="s">
         <v>89</v>
       </c>
       <c r="C86">
         <v>7</v>
       </c>
       <c r="D86" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
+      <c r="A87" s="1">
         <v>11123</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="B87" s="1" t="s">
         <v>90</v>
       </c>
       <c r="C87">
         <v>7</v>
       </c>
       <c r="D87" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
+      <c r="A88" s="1">
         <v>9275</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="B88" s="1" t="s">
         <v>91</v>
       </c>
       <c r="C88">
         <v>7</v>
       </c>
       <c r="D88" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
+      <c r="A89" s="1">
         <v>9256</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="B89" s="1" t="s">
         <v>92</v>
       </c>
       <c r="C89">
         <v>7</v>
       </c>
       <c r="D89" t="s">
-        <v>45</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
+      <c r="A90" s="1">
+        <v>9239</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C90">
+        <v>7</v>
+      </c>
+      <c r="D90" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
+      <c r="A91" s="1">
+        <v>9205</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C91">
+        <v>7</v>
+      </c>
+      <c r="D91" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
+      <c r="A92" s="1">
+        <v>10286</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C92">
+        <v>7</v>
+      </c>
+      <c r="D92" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
+      <c r="A93" s="1">
+        <v>10243</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C93">
+        <v>7</v>
+      </c>
+      <c r="D93" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
+      <c r="A94" s="1">
+        <v>11464</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C94">
+        <v>7</v>
+      </c>
+      <c r="D94" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
+      <c r="A95" s="1">
+        <v>11662</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C95">
+        <v>7</v>
+      </c>
+      <c r="D95" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
+      <c r="A96" s="1">
+        <v>10050</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C96">
+        <v>7</v>
+      </c>
+      <c r="D96" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
+      <c r="A97" s="1">
+        <v>10328</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C97">
+        <v>7</v>
+      </c>
+      <c r="D97" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4">
+      <c r="A98" s="1">
+        <v>9225</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C98">
+        <v>7</v>
+      </c>
+      <c r="D98" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4">
+      <c r="A99" s="1">
+        <v>9265</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C99">
+        <v>7</v>
+      </c>
+      <c r="D99" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4">
+      <c r="A100" s="1">
+        <v>11087</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C100">
+        <v>7</v>
+      </c>
+      <c r="D100" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4">
+      <c r="A101" s="1">
+        <v>9278</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C101">
+        <v>7</v>
+      </c>
+      <c r="D101" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4">
+      <c r="A102" s="1">
+        <v>11629</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C102">
+        <v>7</v>
+      </c>
+      <c r="D102" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4">
+      <c r="A103" s="1">
+        <v>9518</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C103">
+        <v>7</v>
+      </c>
+      <c r="D103" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4">
+      <c r="A104" s="1">
+        <v>9211</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C104">
+        <v>7</v>
+      </c>
+      <c r="D104" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4">
+      <c r="A105" s="1">
+        <v>11699</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C105">
+        <v>7</v>
+      </c>
+      <c r="D105" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4">
+      <c r="A106" s="1">
+        <v>11433</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C106">
+        <v>7</v>
+      </c>
+      <c r="D106" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4">
+      <c r="A107" s="1">
+        <v>11572</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C107">
+        <v>7</v>
+      </c>
+      <c r="D107" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4">
+      <c r="A108" s="1">
+        <v>11682</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C108">
+        <v>7</v>
+      </c>
+      <c r="D108" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4">
+      <c r="A109" s="1">
+        <v>11295</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C109">
+        <v>7</v>
+      </c>
+      <c r="D109" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4">
+      <c r="A110" s="1">
+        <v>10797</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C110">
+        <v>7</v>
+      </c>
+      <c r="D110" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4">
+      <c r="A111" s="1">
+        <v>11401</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C111">
+        <v>7</v>
+      </c>
+      <c r="D111" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4">
+      <c r="A112" s="1">
+        <v>9318</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C112">
+        <v>7</v>
+      </c>
+      <c r="D112" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4">
+      <c r="A113" s="1">
+        <v>9263</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C113">
+        <v>7</v>
+      </c>
+      <c r="D113" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4">
+      <c r="A114" s="1">
+        <v>9274</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C114">
+        <v>7</v>
+      </c>
+      <c r="D114" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4">
+      <c r="A115" s="1">
+        <v>10000</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C115">
+        <v>7</v>
+      </c>
+      <c r="D115" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4">
+      <c r="A116" s="1">
+        <v>9820</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C116">
+        <v>7</v>
+      </c>
+      <c r="D116" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4">
+      <c r="A117" s="1">
+        <v>11207</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C117">
+        <v>7</v>
+      </c>
+      <c r="D117" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4">
+      <c r="A118" s="1">
+        <v>9436</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C118">
+        <v>7</v>
+      </c>
+      <c r="D118" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4">
+      <c r="A119" s="1">
+        <v>9273</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C119">
+        <v>7</v>
+      </c>
+      <c r="D119" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4">
+      <c r="A120" s="1">
+        <v>10479</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C120">
+        <v>7</v>
+      </c>
+      <c r="D120" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4">
+      <c r="A121" s="1">
+        <v>9257</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C121">
+        <v>7</v>
+      </c>
+      <c r="D121" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4">
+      <c r="A122" s="1">
+        <v>9300</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C122">
+        <v>7</v>
+      </c>
+      <c r="D122" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4">
+      <c r="A123" s="1">
+        <v>9244</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C123">
+        <v>7</v>
+      </c>
+      <c r="D123" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4">
+      <c r="A124" s="1">
+        <v>11100</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C124">
+        <v>7</v>
+      </c>
+      <c r="D124" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4">
+      <c r="A125" s="1">
+        <v>9208</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C125">
+        <v>7</v>
+      </c>
+      <c r="D125" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4">
+      <c r="A126" s="1">
+        <v>9299</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C126">
+        <v>7</v>
+      </c>
+      <c r="D126" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4">
+      <c r="A127" s="1">
+        <v>9226</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C127">
+        <v>7</v>
+      </c>
+      <c r="D127" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4">
+      <c r="A128" s="1">
+        <v>11305</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C128">
+        <v>7</v>
+      </c>
+      <c r="D128" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4">
+      <c r="A129" s="1">
+        <v>10220</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C129">
+        <v>7</v>
+      </c>
+      <c r="D129" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4">
+      <c r="A130" s="1">
+        <v>10741</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C130">
+        <v>7</v>
+      </c>
+      <c r="D130" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4">
+      <c r="A131" s="1">
+        <v>10767</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C131">
+        <v>7</v>
+      </c>
+      <c r="D131" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4">
+      <c r="A132" s="1">
+        <v>11585</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C132">
+        <v>7</v>
+      </c>
+      <c r="D132" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4">
+      <c r="A133" s="1">
+        <v>10814</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C133">
+        <v>7</v>
+      </c>
+      <c r="D133" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4">
+      <c r="A134" s="1">
+        <v>10799</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C134">
+        <v>7</v>
+      </c>
+      <c r="D134" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4">
+      <c r="A135" s="1">
+        <v>11244</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C135">
+        <v>7</v>
+      </c>
+      <c r="D135" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4">
+      <c r="A136" s="1">
+        <v>9342</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C136">
+        <v>7</v>
+      </c>
+      <c r="D136" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4">
+      <c r="A137" s="1">
+        <v>10743</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C137">
+        <v>7</v>
+      </c>
+      <c r="D137" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4">
+      <c r="A138" s="1">
+        <v>10154</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C138">
+        <v>7</v>
+      </c>
+      <c r="D138" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4">
+      <c r="A139" s="1">
+        <v>11651</v>
+      </c>
+      <c r="B139" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C139">
+        <v>7</v>
+      </c>
+      <c r="D139" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4">
+      <c r="A140" s="1">
+        <v>8986</v>
+      </c>
+      <c r="B140" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C140">
+        <v>7</v>
+      </c>
+      <c r="D140" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4">
+      <c r="A141" s="1">
+        <v>10407</v>
+      </c>
+      <c r="B141" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C141">
+        <v>7</v>
+      </c>
+      <c r="D141" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4">
+      <c r="A142" s="1">
+        <v>11656</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C142">
+        <v>7</v>
+      </c>
+      <c r="D142" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4">
+      <c r="A143" s="1">
+        <v>11403</v>
+      </c>
+      <c r="B143" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C143">
+        <v>7</v>
+      </c>
+      <c r="D143" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4">
+      <c r="A144" s="1">
+        <v>9230</v>
+      </c>
+      <c r="B144" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C144">
+        <v>7</v>
+      </c>
+      <c r="D144" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4">
+      <c r="A145" s="1">
+        <v>10451</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C145">
+        <v>7</v>
+      </c>
+      <c r="D145" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4">
+      <c r="A146" s="1">
+        <v>9841</v>
+      </c>
+      <c r="B146" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C146">
+        <v>7</v>
+      </c>
+      <c r="D146" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4">
+      <c r="A147" s="1">
+        <v>9235</v>
+      </c>
+      <c r="B147" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C147">
+        <v>7</v>
+      </c>
+      <c r="D147" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4">
+      <c r="A148" s="1">
+        <v>10518</v>
+      </c>
+      <c r="B148" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C148">
+        <v>7</v>
+      </c>
+      <c r="D148" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4">
+      <c r="A149" s="1">
+        <v>11672</v>
+      </c>
+      <c r="B149" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C149">
+        <v>7</v>
+      </c>
+      <c r="D149" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4">
+      <c r="A150" s="1">
+        <v>9261</v>
+      </c>
+      <c r="B150" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C150">
+        <v>7</v>
+      </c>
+      <c r="D150" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4">
+      <c r="A151" s="1">
+        <v>11594</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C151">
+        <v>7</v>
+      </c>
+      <c r="D151" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4">
+      <c r="A152" s="1">
+        <v>9660</v>
+      </c>
+      <c r="B152" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C152">
+        <v>7</v>
+      </c>
+      <c r="D152" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4">
+      <c r="A153" s="1">
+        <v>9937</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C153">
+        <v>7</v>
+      </c>
+      <c r="D153" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4">
+      <c r="A154" s="1">
+        <v>9228</v>
+      </c>
+      <c r="B154" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C154">
+        <v>7</v>
+      </c>
+      <c r="D154" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4">
+      <c r="A155" s="1">
+        <v>11588</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C155">
+        <v>7</v>
+      </c>
+      <c r="D155" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4">
+      <c r="A156" s="1">
+        <v>9216</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C156">
+        <v>7</v>
+      </c>
+      <c r="D156" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4">
+      <c r="A157" s="1">
+        <v>9979</v>
+      </c>
+      <c r="B157" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C157">
+        <v>7</v>
+      </c>
+      <c r="D157" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4">
+      <c r="A158" s="1">
+        <v>11695</v>
+      </c>
+      <c r="B158" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C158">
+        <v>7</v>
+      </c>
+      <c r="D158" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4">
+      <c r="A159" s="1">
+        <v>10357</v>
+      </c>
+      <c r="B159" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C159">
+        <v>7</v>
+      </c>
+      <c r="D159" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4">
+      <c r="A160" s="1">
+        <v>9731</v>
+      </c>
+      <c r="B160" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C160">
+        <v>7</v>
+      </c>
+      <c r="D160" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4">
+      <c r="A161" s="1">
+        <v>9292</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C161">
+        <v>7</v>
+      </c>
+      <c r="D161" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4">
+      <c r="A162" s="1">
+        <v>9930</v>
+      </c>
+      <c r="B162" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C162">
+        <v>7</v>
+      </c>
+      <c r="D162" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4">
+      <c r="A163" s="1">
+        <v>10730</v>
+      </c>
+      <c r="B163" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C163">
+        <v>7</v>
+      </c>
+      <c r="D163" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4">
+      <c r="A164" s="1">
+        <v>11177</v>
+      </c>
+      <c r="B164" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C164">
+        <v>7</v>
+      </c>
+      <c r="D164" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4">
+      <c r="A165" s="1">
+        <v>9237</v>
+      </c>
+      <c r="B165" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C165">
+        <v>7</v>
+      </c>
+      <c r="D165" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4">
+      <c r="A166" s="1">
+        <v>9760</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C166">
+        <v>7</v>
+      </c>
+      <c r="D166" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4">
+      <c r="A167" s="1">
+        <v>11665</v>
+      </c>
+      <c r="B167" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C167">
+        <v>7</v>
+      </c>
+      <c r="D167" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4">
+      <c r="A168" s="1">
+        <v>9220</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C168">
+        <v>7</v>
+      </c>
+      <c r="D168" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4">
+      <c r="A169" s="1">
+        <v>9414</v>
+      </c>
+      <c r="B169" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C169">
+        <v>7</v>
+      </c>
+      <c r="D169" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4">
+      <c r="A170" s="1">
+        <v>9541</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C170">
+        <v>7</v>
+      </c>
+      <c r="D170" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4">
+      <c r="A171" s="1">
+        <v>10816</v>
+      </c>
+      <c r="B171" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C171">
+        <v>7</v>
+      </c>
+      <c r="D171" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4">
+      <c r="A172" s="1">
+        <v>9420</v>
+      </c>
+      <c r="B172" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C172">
+        <v>7</v>
+      </c>
+      <c r="D172" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4">
+      <c r="A173" s="1">
+        <v>9268</v>
+      </c>
+      <c r="B173" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C173">
+        <v>7</v>
+      </c>
+      <c r="D173" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4">
+      <c r="A174" s="1">
+        <v>9303</v>
+      </c>
+      <c r="B174" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C174">
+        <v>7</v>
+      </c>
+      <c r="D174" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: overhaul student interface with premium dark-glass UI, redesign student dashboard, and fix messaging layout issues
</commit_message>
<xml_diff>
--- a/Stdlist.xlsx
+++ b/Stdlist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Apps\Classtest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A86CEF-06CB-47C1-A11E-270F7D578691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A852492C-F991-4199-B9DF-B4317D74C306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{664C5D66-FD01-49D7-B134-66D1304C9B64}"/>
   </bookViews>
@@ -49,13 +49,13 @@
     <t>name</t>
   </si>
   <si>
+    <t>AARZOO GUPTA</t>
+  </si>
+  <si>
     <t>VII</t>
   </si>
   <si>
-    <t>YASH AGRAWAL</t>
-  </si>
-  <si>
-    <t>D</t>
+    <t>B</t>
   </si>
 </sst>
 </file>
@@ -485,426 +485,426 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A2" s="3">
-        <v>11857</v>
+      <c r="A2" s="4">
+        <v>10567</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>5</v>
+      <c r="B2" s="4" t="s">
+        <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
     </row>
     <row r="8" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
     </row>
     <row r="10" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
     </row>
     <row r="11" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
     </row>
     <row r="12" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
     </row>
     <row r="13" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
     </row>
     <row r="14" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
     </row>
     <row r="15" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
     </row>
     <row r="16" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
     </row>
     <row r="17" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
     </row>
     <row r="18" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
     </row>
     <row r="19" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
     </row>
     <row r="20" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
     </row>
     <row r="21" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
     </row>
     <row r="22" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
     </row>
     <row r="23" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
     </row>
     <row r="24" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
     </row>
     <row r="25" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
     </row>
     <row r="26" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
     </row>
     <row r="27" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
     </row>
     <row r="28" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
     </row>
     <row r="29" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
     </row>
     <row r="30" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
     </row>
     <row r="31" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
     </row>
     <row r="32" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
     </row>
     <row r="33" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
     </row>
     <row r="34" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
     </row>
     <row r="35" spans="1:4" ht="15.75" thickBot="1">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
     </row>
     <row r="36" spans="1:4" ht="15.75" thickBot="1">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
     </row>
     <row r="37" spans="1:4" ht="15.75" thickBot="1">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
     </row>
     <row r="38" spans="1:4" ht="15.75" thickBot="1">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4" ht="15.75" thickBot="1">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" ht="15.75" thickBot="1">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
     </row>
     <row r="41" spans="1:4" ht="15.75" thickBot="1">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
     </row>
     <row r="42" spans="1:4" ht="15.75" thickBot="1">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
     </row>
     <row r="43" spans="1:4" ht="15.75" thickBot="1">
       <c r="A43" s="4"/>
       <c r="B43" s="4"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
     </row>
     <row r="44" spans="1:4" ht="15.75" thickBot="1">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
     </row>
     <row r="45" spans="1:4" ht="15.75" thickBot="1">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
     </row>
     <row r="46" spans="1:4" ht="15.75" thickBot="1">
       <c r="A46" s="4"/>
       <c r="B46" s="4"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
     </row>
     <row r="47" spans="1:4" ht="15.75" thickBot="1">
       <c r="A47" s="4"/>
       <c r="B47" s="4"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
     </row>
     <row r="48" spans="1:4" ht="15.75" thickBot="1">
       <c r="A48" s="4"/>
       <c r="B48" s="4"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
     </row>
     <row r="49" spans="1:4" ht="15.75" thickBot="1">
       <c r="A49" s="4"/>
       <c r="B49" s="4"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
     </row>
     <row r="50" spans="1:4" ht="15.75" thickBot="1">
       <c r="A50" s="4"/>
       <c r="B50" s="4"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
     </row>
     <row r="51" spans="1:4" ht="15.75" thickBot="1">
       <c r="A51" s="4"/>
       <c r="B51" s="4"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
     </row>
     <row r="52" spans="1:4" ht="15.75" thickBot="1">
       <c r="A52" s="4"/>
       <c r="B52" s="4"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
     </row>
     <row r="53" spans="1:4" ht="15.75" thickBot="1">
       <c r="A53" s="4"/>
       <c r="B53" s="4"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
     </row>
     <row r="54" spans="1:4" ht="15.75" thickBot="1">
       <c r="A54" s="4"/>
       <c r="B54" s="4"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
     </row>
     <row r="55" spans="1:4" ht="15.75" thickBot="1">
       <c r="A55" s="4"/>
       <c r="B55" s="4"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
     </row>
     <row r="56" spans="1:4" ht="15.75" thickBot="1">
       <c r="A56" s="4"/>
       <c r="B56" s="4"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
     </row>
     <row r="57" spans="1:4" ht="15.75" thickBot="1">
       <c r="A57" s="4"/>
       <c r="B57" s="4"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
     </row>
     <row r="58" spans="1:4" ht="15.75" thickBot="1">
       <c r="A58" s="4"/>
       <c r="B58" s="4"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="3"/>
     </row>
     <row r="59" spans="1:4" ht="15.75" thickBot="1">
       <c r="A59" s="4"/>
       <c r="B59" s="4"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
     </row>
     <row r="60" spans="1:4" ht="15.75" thickBot="1">
       <c r="A60" s="4"/>
       <c r="B60" s="4"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
     </row>
     <row r="61" spans="1:4" ht="15.75" thickBot="1">
       <c r="A61" s="4"/>
       <c r="B61" s="4"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
+      <c r="C61" s="3"/>
+      <c r="D61" s="3"/>
     </row>
     <row r="62" spans="1:4" ht="15.75" thickBot="1">
       <c r="A62" s="4"/>
       <c r="B62" s="4"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
+      <c r="C62" s="3"/>
+      <c r="D62" s="3"/>
     </row>
     <row r="63" spans="1:4" ht="15.75" thickBot="1">
       <c r="A63" s="4"/>
       <c r="B63" s="4"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
     </row>
     <row r="64" spans="1:4" ht="15.75" thickBot="1">
       <c r="A64" s="4"/>
       <c r="B64" s="4"/>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
     </row>
     <row r="65" spans="1:4" ht="15.75" thickBot="1">
       <c r="A65" s="4"/>
       <c r="B65" s="4"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3"/>
     </row>
     <row r="66" spans="1:4" ht="15.75" thickBot="1">
       <c r="A66" s="4"/>
       <c r="B66" s="4"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
     </row>
     <row r="67" spans="1:4" ht="15.75" thickBot="1">
       <c r="A67" s="4"/>
       <c r="B67" s="4"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
+      <c r="C67" s="3"/>
+      <c r="D67" s="3"/>
     </row>
     <row r="68" spans="1:4" ht="15.75" thickBot="1">
       <c r="A68" s="4"/>
       <c r="B68" s="4"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
+      <c r="C68" s="3"/>
+      <c r="D68" s="3"/>
     </row>
     <row r="69" spans="1:4" ht="15.75" thickBot="1">
       <c r="A69" s="4"/>
       <c r="B69" s="4"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
+      <c r="C69" s="3"/>
+      <c r="D69" s="3"/>
     </row>
     <row r="70" spans="1:4" ht="15.75" thickBot="1">
       <c r="A70" s="4"/>
       <c r="B70" s="4"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
     </row>
     <row r="71" spans="1:4" ht="15.75" thickBot="1">
       <c r="A71" s="4"/>

</xml_diff>

<commit_message>
feat: enable HTML file uploads for study notes alongside PDF
</commit_message>
<xml_diff>
--- a/Stdlist.xlsx
+++ b/Stdlist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Apps\Classtest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A852492C-F991-4199-B9DF-B4317D74C306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADCB5DF2-3369-4D5C-BEA9-418B4C0E3F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{664C5D66-FD01-49D7-B134-66D1304C9B64}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="44">
   <si>
     <t>class</t>
   </si>
@@ -49,13 +49,124 @@
     <t>name</t>
   </si>
   <si>
-    <t>AARZOO GUPTA</t>
-  </si>
-  <si>
-    <t>VII</t>
-  </si>
-  <si>
     <t>B</t>
+  </si>
+  <si>
+    <t>AARADHYA SINGH</t>
+  </si>
+  <si>
+    <t>ADITYA</t>
+  </si>
+  <si>
+    <t>ADITYA VASHISTHA</t>
+  </si>
+  <si>
+    <t>AKSHITA DAGUR</t>
+  </si>
+  <si>
+    <t>ANUSHKA SHARMA</t>
+  </si>
+  <si>
+    <t>ANWESHA BARLA</t>
+  </si>
+  <si>
+    <t>APARNA SINGH</t>
+  </si>
+  <si>
+    <t>ARCHIT ARKH</t>
+  </si>
+  <si>
+    <t>ARNAV RAI</t>
+  </si>
+  <si>
+    <t>GAUHAR ALI KHAN</t>
+  </si>
+  <si>
+    <t>HARSHIT CHANDRA</t>
+  </si>
+  <si>
+    <t>ISHAN SAINI</t>
+  </si>
+  <si>
+    <t>JANVI SINGH</t>
+  </si>
+  <si>
+    <t>JAY GAUTAM</t>
+  </si>
+  <si>
+    <t>KRITI GUPTA</t>
+  </si>
+  <si>
+    <t>KUNAL VERMA</t>
+  </si>
+  <si>
+    <t>KUSHAGRA RAWAT</t>
+  </si>
+  <si>
+    <t>LEENA SINGH</t>
+  </si>
+  <si>
+    <t>MANYA KUMARI</t>
+  </si>
+  <si>
+    <t>MOHIT SHARMA</t>
+  </si>
+  <si>
+    <t>NAVYA AGRAWAL</t>
+  </si>
+  <si>
+    <t>NIKHIL SAINI</t>
+  </si>
+  <si>
+    <t>NIMISHA DESHWAR</t>
+  </si>
+  <si>
+    <t>NIRANJAN PARASHAR</t>
+  </si>
+  <si>
+    <t>NUZHAT KHAN</t>
+  </si>
+  <si>
+    <t>PAARTH SHARMA</t>
+  </si>
+  <si>
+    <t>PIYUSH PATASARIYA</t>
+  </si>
+  <si>
+    <t>PRACHI SINGH</t>
+  </si>
+  <si>
+    <t>PRAGYAN RANA</t>
+  </si>
+  <si>
+    <t>PRASUN RANA</t>
+  </si>
+  <si>
+    <t>PRATYUSH THENUA</t>
+  </si>
+  <si>
+    <t>RAGHAV KAUSHIK</t>
+  </si>
+  <si>
+    <t>SATWIK TIWARI</t>
+  </si>
+  <si>
+    <t>SHASHWAT SHARMA</t>
+  </si>
+  <si>
+    <t>SUSHANT VERMA</t>
+  </si>
+  <si>
+    <t>TEJAS PARASHAR</t>
+  </si>
+  <si>
+    <t>TRISHA SINHA</t>
+  </si>
+  <si>
+    <t>VANSH CHATURVEDI</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
@@ -486,239 +597,535 @@
     </row>
     <row r="2" spans="1:4" ht="15.75" thickBot="1">
       <c r="A2" s="4">
-        <v>10567</v>
+        <v>8794</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A3" s="4">
+        <v>11445</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
+      <c r="C3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="A4" s="4">
+        <v>10443</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
+      <c r="A5" s="4">
+        <v>11550</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+      <c r="A6" s="4">
+        <v>8757</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
+      <c r="A7" s="4">
+        <v>11114</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="A8" s="4">
+        <v>9989</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="A9" s="4">
+        <v>9382</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
+      <c r="A10" s="4">
+        <v>10100</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
+      <c r="A11" s="4">
+        <v>11282</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="12" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+      <c r="A12" s="4">
+        <v>8762</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="A13" s="4">
+        <v>9031</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="14" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
+      <c r="A14" s="4">
+        <v>11582</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
+      <c r="A15" s="4">
+        <v>8692</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="16" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
+      <c r="A16" s="4">
+        <v>8646</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="17" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
+      <c r="A17" s="4">
+        <v>9606</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="18" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
+      <c r="A18" s="4">
+        <v>10511</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
+      <c r="A19" s="4">
+        <v>8687</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="20" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
+      <c r="A20" s="4">
+        <v>8793</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="21" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
+      <c r="A21" s="4">
+        <v>8697</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="22" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
+      <c r="A22" s="4">
+        <v>11558</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="23" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
+      <c r="A23" s="4">
+        <v>8637</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="24" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
+      <c r="A24" s="4">
+        <v>9842</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="25" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
+      <c r="A25" s="4">
+        <v>8870</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="26" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
+      <c r="A26" s="4">
+        <v>9355</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
+      <c r="A27" s="4">
+        <v>10669</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="28" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
+      <c r="A28" s="4">
+        <v>8747</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="29" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
+      <c r="A29" s="4">
+        <v>11238</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="30" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
+      <c r="A30" s="4">
+        <v>11527</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="31" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A31" s="4"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
+      <c r="A31" s="4">
+        <v>11528</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="32" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
+      <c r="A32" s="4">
+        <v>11590</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="33" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
+      <c r="A33" s="4">
+        <v>8766</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="34" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
+      <c r="A34" s="4">
+        <v>8749</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="35" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
+      <c r="A35" s="4">
+        <v>9614</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="36" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
+      <c r="A36" s="4">
+        <v>8644</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="37" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
+      <c r="A37" s="4">
+        <v>11022</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="38" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
+      <c r="A38" s="4">
+        <v>8642</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="39" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A39" s="4"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
+      <c r="A39" s="4">
+        <v>9623</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="40" spans="1:4" ht="15.75" thickBot="1">
       <c r="A40" s="4"/>

</xml_diff>